<commit_message>
feat: add Sheet ⑥ for institutional-access PDF download tracking (54 papers)
- New tab lists 54 non-OA papers requiring institutional access
- Includes DOI hyperlinks, publisher info, and check column (✅/❌/🔍)
- Remaining 74 papers are Gold/Hybrid/Bronze OA (freely accessible)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resource/TCS_screening_coding_v1.xlsx
+++ b/resource/TCS_screening_coding_v1.xlsx
@@ -12,9 +12,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="③ Full-text 코딩" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="④ 전체현황" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑤ 코딩가이드" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="⑥ 기관접근 필요 (PDF)" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'① T_A 스크리닝 (799건)'!$A$2:$K$801</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'⑥ 기관접근 필요 (PDF)'!$A$2:$H$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,8 +83,23 @@
       <b val="1"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00FF0000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -141,6 +158,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
         <bgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+        <bgColor rgb="00C00000"/>
       </patternFill>
     </fill>
   </fills>
@@ -214,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -343,6 +366,24 @@
     <xf numFmtId="0" fontId="3" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -43470,39 +43511,17 @@
       <c r="A3" s="46" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="46" t="inlineStr">
-        <is>
-          <t>SCOPUS_78</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="inlineStr">
-        <is>
-          <t>A TCCM-Based Systematic Literature Review of Anthropomorphism in Human-AI Interaction and Future Research Agenda</t>
-        </is>
-      </c>
-      <c r="D3" s="46" t="n">
-        <v>2026</v>
-      </c>
-      <c r="E3" s="46" t="inlineStr">
-        <is>
-          <t>Journal of Technology in Behavioral Science</t>
-        </is>
-      </c>
-      <c r="F3" s="47" t="inlineStr">
-        <is>
-          <t>📄</t>
-        </is>
-      </c>
-      <c r="G3" s="46" t="inlineStr">
-        <is>
-          <t>Ansari, B.; Sameer, A.</t>
-        </is>
-      </c>
-      <c r="H3" s="46" t="n"/>
-      <c r="I3" s="46" t="n"/>
-      <c r="J3" s="46" t="n"/>
-      <c r="K3" s="46" t="n"/>
-      <c r="L3" s="46" t="n"/>
+      <c r="B3" s="10" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="10" t="n"/>
+      <c r="H3" s="10" t="n"/>
+      <c r="I3" s="10" t="n"/>
+      <c r="J3" s="10" t="n"/>
+      <c r="K3" s="10" t="n"/>
+      <c r="L3" s="11" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="46" t="n">
@@ -48343,7 +48362,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
@@ -49780,4 +49799,1904 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="51" t="inlineStr">
+        <is>
+          <t>📥 기관 접근 필요 — PDF 다운로드 대상 (54편)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="52" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="52" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C2" s="52" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D2" s="52" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E2" s="52" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F2" s="52" t="inlineStr">
+        <is>
+          <t>DOI Link</t>
+        </is>
+      </c>
+      <c r="G2" s="52" t="inlineStr">
+        <is>
+          <t>Publisher</t>
+        </is>
+      </c>
+      <c r="H2" s="52" t="inlineStr">
+        <is>
+          <t>✅ 확보</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="53" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_78</t>
+        </is>
+      </c>
+      <c r="C3" s="53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>A TCCM-Based Systematic Literature Review of Anthropomorphism in Human-AI Interaction and Future Research Agenda</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Technology in Behavioral Science</t>
+        </is>
+      </c>
+      <c r="F3" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s41347-026-00594-7</t>
+        </is>
+      </c>
+      <c r="G3" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H3" s="55" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="53" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_24</t>
+        </is>
+      </c>
+      <c r="C4" s="53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Beyond Substitution: How Teacher Interpersonal Behaviours Empower Students to Communicate With AI—A Dual-Mediation Model of Enjoyment and Trust</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>European Journal of Education</t>
+        </is>
+      </c>
+      <c r="F4" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/ejed.70499</t>
+        </is>
+      </c>
+      <c r="G4" s="53" t="inlineStr"/>
+      <c r="H4" s="55" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_48</t>
+        </is>
+      </c>
+      <c r="C5" s="53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>From Prompts to Dependency: Standardization of the AI Chatbot Dependence Scale In A Turkish Context And Associations With Big Five Personality Traits</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Human-Computer Interaction</t>
+        </is>
+      </c>
+      <c r="F5" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/10447318.2026.2629519</t>
+        </is>
+      </c>
+      <c r="G5" s="53" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H5" s="55" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_21</t>
+        </is>
+      </c>
+      <c r="C6" s="53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>In AI We Trust? Exploring the Role of Explainable GenAI and Expertise in Education</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>Human Factors</t>
+        </is>
+      </c>
+      <c r="F6" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/00187208251401773</t>
+        </is>
+      </c>
+      <c r="G6" s="53" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H6" s="55" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_26</t>
+        </is>
+      </c>
+      <c r="C7" s="53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Trusting the Machine: How AI Assessment Feedback and AI Literacy Shape Students' Idea Implementation Skills</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>European Journal of Education</t>
+        </is>
+      </c>
+      <c r="F7" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/ejed.70457</t>
+        </is>
+      </c>
+      <c r="G7" s="53" t="inlineStr"/>
+      <c r="H7" s="55" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="53" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_36</t>
+        </is>
+      </c>
+      <c r="C8" s="53" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>‘ChatGPT can make mistakes’ warnings fail: A randomized controlled trial</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Medical Education</t>
+        </is>
+      </c>
+      <c r="F8" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/medu.70056</t>
+        </is>
+      </c>
+      <c r="G8" s="53" t="inlineStr"/>
+      <c r="H8" s="55" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>WOS_130</t>
+        </is>
+      </c>
+      <c r="C9" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>A comprehensive structural equation modeling analysis of factors influencing teacher acceptance of AI in education through an extended TAM framework</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>EDUCATION AND INFORMATION TECHNOLOGIES</t>
+        </is>
+      </c>
+      <c r="F9" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10639-025-13833-w</t>
+        </is>
+      </c>
+      <c r="G9" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H9" s="55" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="53" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="46" t="inlineStr">
+        <is>
+          <t>WOS_63</t>
+        </is>
+      </c>
+      <c r="C10" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>ARTIFICIAL INTELLIGENCE (AI) LITERACY AMONG TEACHERS: THE CASE OF ITMO UNI-VERSITY</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>REVISTA CONRADO</t>
+        </is>
+      </c>
+      <c r="F10" s="56" t="inlineStr">
+        <is>
+          <t>(DOI 없음 — 수동 검색 필요)</t>
+        </is>
+      </c>
+      <c r="G10" s="53" t="inlineStr"/>
+      <c r="H10" s="55" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_251</t>
+        </is>
+      </c>
+      <c r="C11" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence as a Catalyst for Promoting Utility Value Perceptions of Chemistry</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Chemical Education</t>
+        </is>
+      </c>
+      <c r="F11" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1021/acs.jchemed.5c00625</t>
+        </is>
+      </c>
+      <c r="G11" s="53" t="inlineStr"/>
+      <c r="H11" s="55" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_492</t>
+        </is>
+      </c>
+      <c r="C12" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Building Trust in AI Through Dialogues With Eastern Ethics: Toward Ethical Partnerships in Education</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Learning Technologies</t>
+        </is>
+      </c>
+      <c r="F12" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tlt.2025.3604616</t>
+        </is>
+      </c>
+      <c r="G12" s="53" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="H12" s="55" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="53" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_293</t>
+        </is>
+      </c>
+      <c r="C13" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Can Generative Artificial Intelligence be a Good Teaching Assistant?—An Empirical Analysis Based on Generative AI-Assisted Teaching</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Computer Assisted Learning</t>
+        </is>
+      </c>
+      <c r="F13" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jcal.70027</t>
+        </is>
+      </c>
+      <c r="G13" s="53" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H13" s="55" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="53" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_240</t>
+        </is>
+      </c>
+      <c r="C14" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Can student accurately identify artificial intelligence generated content? an exploration of AIGC credibility from user perspective in education</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>Education and Information Technologies</t>
+        </is>
+      </c>
+      <c r="F14" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10639-025-13448-1</t>
+        </is>
+      </c>
+      <c r="G14" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H14" s="55" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="53" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_449</t>
+        </is>
+      </c>
+      <c r="C15" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>Cognitive Risks of AI: Literacy, Trust, and Critical Thinking</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Computer Information Systems</t>
+        </is>
+      </c>
+      <c r="F15" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/08874417.2025.2582050</t>
+        </is>
+      </c>
+      <c r="G15" s="53" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H15" s="55" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="53" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" s="46" t="inlineStr">
+        <is>
+          <t>WOS_58</t>
+        </is>
+      </c>
+      <c r="C16" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>Demystifying School Leader Career Sustainability: The Role of Trust in Artificial Intelligence and Artificial Intelligence Collaboration</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>JOURNAL OF COMPUTER ASSISTED LEARNING</t>
+        </is>
+      </c>
+      <c r="F16" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jcal.70135</t>
+        </is>
+      </c>
+      <c r="G16" s="53" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H16" s="55" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="53" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" s="46" t="inlineStr">
+        <is>
+          <t>WOS_65</t>
+        </is>
+      </c>
+      <c r="C17" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>Engineering Students' Use of Large Language Model Tools: An Empirical Study Based on a Survey of Students from 12 Universities</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>EDUCATION SCIENCES</t>
+        </is>
+      </c>
+      <c r="F17" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/educsci15030280</t>
+        </is>
+      </c>
+      <c r="G17" s="53" t="inlineStr">
+        <is>
+          <t>MDPI</t>
+        </is>
+      </c>
+      <c r="H17" s="55" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="53" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_538</t>
+        </is>
+      </c>
+      <c r="C18" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>English language teachers' perspectives on digital trust in AI-supported education</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>British Educational Research Journal</t>
+        </is>
+      </c>
+      <c r="F18" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/berj.4209</t>
+        </is>
+      </c>
+      <c r="G18" s="53" t="inlineStr"/>
+      <c r="H18" s="55" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="53" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_37</t>
+        </is>
+      </c>
+      <c r="C19" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Enhancing college students’ ai literacy through human-ai co-creation: A quantitative study</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Interactive Learning Environments</t>
+        </is>
+      </c>
+      <c r="F19" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/10494820.2025.2495733</t>
+        </is>
+      </c>
+      <c r="G19" s="53" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H19" s="55" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="53" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="46" t="inlineStr">
+        <is>
+          <t>WOS_129</t>
+        </is>
+      </c>
+      <c r="C20" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Extending the technology acceptance model: The role of subjective norms, ethics, and trust in AI tool adoption among students</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>COMPUTERS AND EDUCATION: ARTIFICIAL INTELLIGENCE</t>
+        </is>
+      </c>
+      <c r="F20" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.caeai.2025.100379</t>
+        </is>
+      </c>
+      <c r="G20" s="53" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H20" s="55" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="53" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="46" t="inlineStr">
+        <is>
+          <t>WOS_175</t>
+        </is>
+      </c>
+      <c r="C21" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Fostering AI literacy in pre-service teachers: impact of a training intervention on awareness, attitude and trust in AI</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>FRONTIERS IN EDUCATION</t>
+        </is>
+      </c>
+      <c r="F21" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3389/feduc.2025.1668078</t>
+        </is>
+      </c>
+      <c r="G21" s="53" t="inlineStr"/>
+      <c r="H21" s="55" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="53" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_142</t>
+        </is>
+      </c>
+      <c r="C22" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>From classroom to Boardroom: Ethical and cognitive challenges of ChatGPT use among DBA students in business problem-solving</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Management Education</t>
+        </is>
+      </c>
+      <c r="F22" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ijme.2025.101254</t>
+        </is>
+      </c>
+      <c r="G22" s="53" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H22" s="55" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="53" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_298</t>
+        </is>
+      </c>
+      <c r="C23" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>From resistance to acceptance: the dynamics of educators’ intentions to use chatbots and the role of educators’ autocratic behaviour</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Asian Education and Development Studies</t>
+        </is>
+      </c>
+      <c r="F23" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/aeds-06-2024-0134</t>
+        </is>
+      </c>
+      <c r="G23" s="53" t="inlineStr"/>
+      <c r="H23" s="55" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="53" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" s="46" t="inlineStr">
+        <is>
+          <t>WOS_16</t>
+        </is>
+      </c>
+      <c r="C24" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>Higher education students' trust and use of ChatGPT: empirical evidence</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>INTERNATIONAL JOURNAL OF TECHNOLOGY ENHANCED LEARNING</t>
+        </is>
+      </c>
+      <c r="F24" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/ijtel.2024.10061581</t>
+        </is>
+      </c>
+      <c r="G24" s="53" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H24" s="55" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="53" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_426</t>
+        </is>
+      </c>
+      <c r="C25" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>Hooked on help: Student overreliance on ChatGPT in higher education</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Information Technology Teaching Cases</t>
+        </is>
+      </c>
+      <c r="F25" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/20438869251397953</t>
+        </is>
+      </c>
+      <c r="G25" s="53" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H25" s="55" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="53" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_212</t>
+        </is>
+      </c>
+      <c r="C26" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>How Learners’ Trust Changes in Generative AI over a Semester of Undergraduate Courses</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Artificial Intelligence in Education</t>
+        </is>
+      </c>
+      <c r="F26" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s40593-024-00446-6</t>
+        </is>
+      </c>
+      <c r="G26" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H26" s="55" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="53" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_45</t>
+        </is>
+      </c>
+      <c r="C27" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>InquiryGPT: Augmenting ChatGPT for enhancing inquiry-based learning in STEM education</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Educational Computing Research</t>
+        </is>
+      </c>
+      <c r="F27" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/07356331241289824</t>
+        </is>
+      </c>
+      <c r="G27" s="53" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H27" s="55" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="53" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_421</t>
+        </is>
+      </c>
+      <c r="C28" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Investigating the antecedents and consequences of trust in ChatGPT across cultures: a learner-centric perspective</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Internet Research</t>
+        </is>
+      </c>
+      <c r="F28" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/intr-08-2024-1237</t>
+        </is>
+      </c>
+      <c r="G28" s="53" t="inlineStr"/>
+      <c r="H28" s="55" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="53" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_46</t>
+        </is>
+      </c>
+      <c r="C29" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>Knowledge is not all you need for comfort in use of AI in healthcare</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>Public Health</t>
+        </is>
+      </c>
+      <c r="F29" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.puhe.2024.11.019</t>
+        </is>
+      </c>
+      <c r="G29" s="53" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H29" s="55" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="53" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_235</t>
+        </is>
+      </c>
+      <c r="C30" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>Measuring undergraduate students' reliance on Generative AI during problem-solving: Scale development and validation</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Computers and Education</t>
+        </is>
+      </c>
+      <c r="F30" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.compedu.2025.105329</t>
+        </is>
+      </c>
+      <c r="G30" s="53" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H30" s="55" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="53" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="46" t="inlineStr">
+        <is>
+          <t>WOS_180</t>
+        </is>
+      </c>
+      <c r="C31" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>Multi-stakeholder perspective on responsible artificial intelligence and acceptability in education</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>NPJ SCIENCE OF LEARNING</t>
+        </is>
+      </c>
+      <c r="F31" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1038/s41539-025-00333-2</t>
+        </is>
+      </c>
+      <c r="G31" s="53" t="inlineStr"/>
+      <c r="H31" s="55" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="53" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_130</t>
+        </is>
+      </c>
+      <c r="C32" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>Research of Ethical Adoption of College Students' Learning Applications of Generative Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Computer Assisted Learning</t>
+        </is>
+      </c>
+      <c r="F32" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/jcal.70146</t>
+        </is>
+      </c>
+      <c r="G32" s="53" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H32" s="55" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="53" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_315</t>
+        </is>
+      </c>
+      <c r="C33" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>The Review of Studies on Explainable Artificial Intelligence in Educational Research</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Educational Computing Research</t>
+        </is>
+      </c>
+      <c r="F33" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/07356331241310915</t>
+        </is>
+      </c>
+      <c r="G33" s="53" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H33" s="55" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="53" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" s="46" t="inlineStr">
+        <is>
+          <t>WOS_80</t>
+        </is>
+      </c>
+      <c r="C34" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>Trust in AI Feedback: Challenges in Pharmacy Education</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>MEDICAL SCIENCE EDUCATOR</t>
+        </is>
+      </c>
+      <c r="F34" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s40670-025-02440-6</t>
+        </is>
+      </c>
+      <c r="G34" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H34" s="55" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="53" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_424</t>
+        </is>
+      </c>
+      <c r="C35" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>Trust, resistance, and transformation: A Q-methodological study of teachers' perspectives on AI-generated feedback in second language writing</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Foreign Language Annals</t>
+        </is>
+      </c>
+      <c r="F35" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/flan.70042</t>
+        </is>
+      </c>
+      <c r="G35" s="53" t="inlineStr"/>
+      <c r="H35" s="55" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="53" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" s="46" t="inlineStr">
+        <is>
+          <t>WOS_107</t>
+        </is>
+      </c>
+      <c r="C36" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>Understanding teachers' willingness to use artificial intelligence-based teaching analysis system: extending TAM model with teaching efficacy, goal orientation, anxiety, and trust</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>INTERACTIVE LEARNING ENVIRONMENTS</t>
+        </is>
+      </c>
+      <c r="F36" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/10494820.2024.2365345</t>
+        </is>
+      </c>
+      <c r="G36" s="53" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H36" s="55" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="53" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_243</t>
+        </is>
+      </c>
+      <c r="C37" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Understanding the intention to use artificial intelligence chatbots in education: The role of individual innovativeness and AI trust among university students</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Computational Social Science</t>
+        </is>
+      </c>
+      <c r="F37" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s42001-025-00387-7</t>
+        </is>
+      </c>
+      <c r="G37" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H37" s="55" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="53" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_354</t>
+        </is>
+      </c>
+      <c r="C38" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>Unpacking perceived risks and AI trust influences pre-service teachers’ AI acceptance: A structural equation modeling-based multi-group analysis</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Education and Information Technologies</t>
+        </is>
+      </c>
+      <c r="F38" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10639-024-12905-7</t>
+        </is>
+      </c>
+      <c r="G38" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H38" s="55" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="53" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_322</t>
+        </is>
+      </c>
+      <c r="C39" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Unveiling the drivers of ChatGPT utilization in higher education sectors: the direct role of perceived knowledge and the mediating role of trust in ChatGPT</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Education and Information Technologies</t>
+        </is>
+      </c>
+      <c r="F39" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10639-024-13095-y</t>
+        </is>
+      </c>
+      <c r="G39" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H39" s="55" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="53" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_292</t>
+        </is>
+      </c>
+      <c r="C40" s="53" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>Why do graduate students use generative AI in thesis writing? the influence of self-efficacy, time pressure, and trust</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Current Psychology</t>
+        </is>
+      </c>
+      <c r="F40" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s12144-025-08003-7</t>
+        </is>
+      </c>
+      <c r="G40" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H40" s="55" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="53" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_731</t>
+        </is>
+      </c>
+      <c r="C41" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Design and Evaluation of Trustworthy Knowledge Tracing Model for Intelligent Tutoring System</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>IEEE Transactions on Learning Technologies</t>
+        </is>
+      </c>
+      <c r="F41" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1109/tlt.2024.3403135</t>
+        </is>
+      </c>
+      <c r="G41" s="53" t="inlineStr">
+        <is>
+          <t>IEEE</t>
+        </is>
+      </c>
+      <c r="H41" s="55" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="53" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_719</t>
+        </is>
+      </c>
+      <c r="C42" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Evaluating ChatGPT adoption through the lens of the technology acceptance model: perspectives from higher education</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Technological Learning, Innovation and Development</t>
+        </is>
+      </c>
+      <c r="F42" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/ijtlid.2024.140316</t>
+        </is>
+      </c>
+      <c r="G42" s="53" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H42" s="55" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="53" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_630</t>
+        </is>
+      </c>
+      <c r="C43" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Exploring higher education students’ continuance usage intention of ChatGPT: amalgamation of the information system success model and the stimulus-organism-response paradigm</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Information and Learning Technology</t>
+        </is>
+      </c>
+      <c r="F43" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1108/ijilt-01-2024-0006</t>
+        </is>
+      </c>
+      <c r="G43" s="53" t="inlineStr"/>
+      <c r="H43" s="55" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="53" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_53</t>
+        </is>
+      </c>
+      <c r="C44" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>Patients’ attitudes toward the use of artificial intelligence as a diagnostic tool in radiology in Saudi Arabia: Cross-sectional study</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>JMIR Human Factors</t>
+        </is>
+      </c>
+      <c r="F44" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.2196/53108</t>
+        </is>
+      </c>
+      <c r="G44" s="53" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H44" s="55" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="53" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_717</t>
+        </is>
+      </c>
+      <c r="C45" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Students’ Response to ChatGPT: An Adaptive Technology-To-Performance Model</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Computer Information Systems</t>
+        </is>
+      </c>
+      <c r="F45" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/08874417.2024.2386546</t>
+        </is>
+      </c>
+      <c r="G45" s="53" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H45" s="55" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="53" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="46" t="inlineStr">
+        <is>
+          <t>WOS_105</t>
+        </is>
+      </c>
+      <c r="C46" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>TRANSFORMATIVE PEDAGOGY IN THE DIGITAL AGE: UNRAVELING THE IMPACT OF ARTIFICIAL INTELLIGENCE ON HIGHER EDUCATION STUDENTS</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>PROBLEMS OF EDUCATION IN THE 21ST CENTURY</t>
+        </is>
+      </c>
+      <c r="F46" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.33225/pec/24.82.630</t>
+        </is>
+      </c>
+      <c r="G46" s="53" t="inlineStr"/>
+      <c r="H46" s="55" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="53" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_763</t>
+        </is>
+      </c>
+      <c r="C47" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>The Future of Learning: Building Trust and Transparency in AI Education</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Management Practices, Humanities and Social Sciences (JMPHSS)</t>
+        </is>
+      </c>
+      <c r="F47" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.33152/jmphss-8.3.6</t>
+        </is>
+      </c>
+      <c r="G47" s="53" t="inlineStr"/>
+      <c r="H47" s="55" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="53" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_56</t>
+        </is>
+      </c>
+      <c r="C48" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>The effect of artificial intelligence on patient-physician trust: Cross-sectional vignette study</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Medical Internet Research</t>
+        </is>
+      </c>
+      <c r="F48" s="56" t="inlineStr">
+        <is>
+          <t>(DOI 없음 — 수동 검색 필요)</t>
+        </is>
+      </c>
+      <c r="G48" s="53" t="inlineStr"/>
+      <c r="H48" s="55" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="53" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="46" t="inlineStr">
+        <is>
+          <t>WOS_79</t>
+        </is>
+      </c>
+      <c r="C49" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>The effects of over-reliance on AI dialogue systems on students' cognitive abilities: a systematic review</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>SMART LEARNING ENVIRONMENTS</t>
+        </is>
+      </c>
+      <c r="F49" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1186/s40561-024-00316-7</t>
+        </is>
+      </c>
+      <c r="G49" s="53" t="inlineStr"/>
+      <c r="H49" s="55" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="53" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_57</t>
+        </is>
+      </c>
+      <c r="C50" s="53" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>To advance AI use in education, focus on understanding educators</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Artificial Intelligence in Education</t>
+        </is>
+      </c>
+      <c r="F50" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s40593-023-00351-4</t>
+        </is>
+      </c>
+      <c r="G50" s="53" t="inlineStr">
+        <is>
+          <t>Springer</t>
+        </is>
+      </c>
+      <c r="H50" s="55" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="53" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_63</t>
+        </is>
+      </c>
+      <c r="C51" s="53" t="n">
+        <v>2023</v>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Trust or mistrust in algorithmic grading? An embedded agency perspective</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Information Management</t>
+        </is>
+      </c>
+      <c r="F51" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.ijinfomgt.2022.102555</t>
+        </is>
+      </c>
+      <c r="G51" s="53" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H51" s="55" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="53" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_67</t>
+        </is>
+      </c>
+      <c r="C52" s="53" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>Do people favor artificial intelligence over physicians? A survey among the general population and their view on artificial intelligence in medicine</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Value in Health</t>
+        </is>
+      </c>
+      <c r="F52" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.jval.2021.09.004</t>
+        </is>
+      </c>
+      <c r="G52" s="53" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H52" s="55" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_65</t>
+        </is>
+      </c>
+      <c r="C53" s="53" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Incorporating AI and learning analytics to build trustworthy peer assessment systems</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>British Journal of Educational Technology</t>
+        </is>
+      </c>
+      <c r="F53" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/bjet.13233</t>
+        </is>
+      </c>
+      <c r="G53" s="53" t="inlineStr"/>
+      <c r="H53" s="55" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="46" t="inlineStr">
+        <is>
+          <t>SCOPUS_815</t>
+        </is>
+      </c>
+      <c r="C54" s="53" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>Teachable Conversational Agents for Crowdwork: Effects on Performance and Trust</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Proceedings of the ACM on Human-Computer Interaction</t>
+        </is>
+      </c>
+      <c r="F54" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1145/3555223</t>
+        </is>
+      </c>
+      <c r="G54" s="53" t="inlineStr">
+        <is>
+          <t>ACM</t>
+        </is>
+      </c>
+      <c r="H54" s="55" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="53" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" s="46" t="inlineStr">
+        <is>
+          <t>PSYC_69</t>
+        </is>
+      </c>
+      <c r="C55" s="53" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Limits of trust in medical AI</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Journal of Medical Ethics: Journal of the Institute of Medical Ethics</t>
+        </is>
+      </c>
+      <c r="F55" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1136/medethics-2019-105935</t>
+        </is>
+      </c>
+      <c r="G55" s="53" t="inlineStr">
+        <is>
+          <t>BMJ</t>
+        </is>
+      </c>
+      <c r="H55" s="55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="53" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" s="46" t="inlineStr">
+        <is>
+          <t>WOS_50</t>
+        </is>
+      </c>
+      <c r="C56" s="53" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Understanding user trust in artificial intelligence-based educational systems: Evidence from China</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>BRITISH JOURNAL OF EDUCATIONAL TECHNOLOGY</t>
+        </is>
+      </c>
+      <c r="F56" s="54" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/bjet.12994</t>
+        </is>
+      </c>
+      <c r="G56" s="53" t="inlineStr"/>
+      <c r="H56" s="55" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:H56"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="H3:H56" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="✅(확보), ❌(불가), 🔍(검색중)" type="list">
+      <formula1>"✅,❌,🔍"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F37" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F38" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F39" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F40" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F41" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F42" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F43" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F44" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F45" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F46" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F47" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F53" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId52"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add 23 failed OA papers to Sheet ⑥ and OA download infrastructure
- Sheet ⑥ updated: 54 non-OA + 23 OA download failures = 77 manual download targets
- Added OA PDF download script (Unpaywall, Semantic Scholar, OpenAlex)
- 51/74 OA papers downloaded successfully (49.4 MB)
- 23 papers blocked by publisher bot protection (Wiley 9, Elsevier 7, SAGE 3, T&F 2, other 2)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resource/TCS_screening_coding_v1.xlsx
+++ b/resource/TCS_screening_coding_v1.xlsx
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -98,8 +98,25 @@
       <color rgb="00FF0000"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00E65100"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -166,8 +183,26 @@
         <bgColor rgb="00C00000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFE0B2"/>
+        <bgColor rgb="00FFE0B2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFB74D"/>
+        <bgColor rgb="00FFB74D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF3E0"/>
+        <bgColor rgb="00FFF3E0"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -233,11 +268,17 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -385,6 +426,20 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -49807,7 +49862,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H56"/>
+  <dimension ref="A1:H82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -49823,7 +49878,7 @@
     <row r="1">
       <c r="A1" s="51" t="inlineStr">
         <is>
-          <t>📥 기관 접근 필요 — PDF 다운로드 대상 (54편)</t>
+          <t>📥 수동 다운로드 필요 — 비OA 54편 + OA 실패 23편 = 총 77편</t>
         </is>
       </c>
     </row>
@@ -51633,9 +51688,841 @@
       <c r="G56" s="53" t="inlineStr"/>
       <c r="H56" s="55" t="inlineStr"/>
     </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="57" t="inlineStr">
+        <is>
+          <t>📥 OA 논문 중 자동 다운로드 실패 — 수동 다운로드 필요 (23편)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="58" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B59" s="58" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="C59" s="58" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D59" s="58" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E59" s="58" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F59" s="58" t="inlineStr">
+        <is>
+          <t>DOI Link</t>
+        </is>
+      </c>
+      <c r="G59" s="58" t="inlineStr">
+        <is>
+          <t>Publisher</t>
+        </is>
+      </c>
+      <c r="H59" s="58" t="inlineStr">
+        <is>
+          <t>✅ 확보</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="B60" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_12</t>
+        </is>
+      </c>
+      <c r="C60" s="59" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D60" s="61" t="inlineStr">
+        <is>
+          <t>Generative AI in higher education: Ethical and behavioral factors influencing students’ intentions to use ChatGPT</t>
+        </is>
+      </c>
+      <c r="E60" s="61" t="inlineStr">
+        <is>
+          <t>Computers and Education Open</t>
+        </is>
+      </c>
+      <c r="F60" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.caeo.2026.100336</t>
+        </is>
+      </c>
+      <c r="G60" s="59" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H60" s="59" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="B61" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_126</t>
+        </is>
+      </c>
+      <c r="C61" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D61" s="61" t="inlineStr">
+        <is>
+          <t>Uncovering the Mediating Effects of AI Trust and Self-Efficacy on Engagement in Human-GenAI Communication for EFL Learning</t>
+        </is>
+      </c>
+      <c r="E61" s="61" t="inlineStr">
+        <is>
+          <t>European Journal of Education</t>
+        </is>
+      </c>
+      <c r="F61" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/ejed.70336</t>
+        </is>
+      </c>
+      <c r="G61" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H61" s="59" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="B62" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_140</t>
+        </is>
+      </c>
+      <c r="C62" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D62" s="61" t="inlineStr">
+        <is>
+          <t>Factors influencing intention to adopt an AI chatbot for learning in higher education: An integrated PLS-SEM, IPMA, and ANN approach</t>
+        </is>
+      </c>
+      <c r="E62" s="61" t="inlineStr">
+        <is>
+          <t>Computers and Education: Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F62" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.caeai.2025.100477</t>
+        </is>
+      </c>
+      <c r="G62" s="59" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H62" s="59" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="B63" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_143</t>
+        </is>
+      </c>
+      <c r="C63" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D63" s="61" t="inlineStr">
+        <is>
+          <t>Can Adopt AI-Powered Educational Technology Buffer Against Academic Stress and School Burnout? A Protective Model Proposal</t>
+        </is>
+      </c>
+      <c r="E63" s="61" t="inlineStr">
+        <is>
+          <t>Psychology in the Schools</t>
+        </is>
+      </c>
+      <c r="F63" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1002/pits.70068</t>
+        </is>
+      </c>
+      <c r="G63" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H63" s="59" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="B64" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_190</t>
+        </is>
+      </c>
+      <c r="C64" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D64" s="61" t="inlineStr">
+        <is>
+          <t>Critical Thinking as a Key to Empowering Graduate Students’ English Learning in the AI Era</t>
+        </is>
+      </c>
+      <c r="E64" s="61" t="inlineStr">
+        <is>
+          <t>SAGE Open</t>
+        </is>
+      </c>
+      <c r="F64" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/21582440251399104</t>
+        </is>
+      </c>
+      <c r="G64" s="59" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H64" s="59" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="B65" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_229</t>
+        </is>
+      </c>
+      <c r="C65" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D65" s="61" t="inlineStr">
+        <is>
+          <t>The role of critical thinking on undergraduates' reliance behaviours on generative AI in problem-solving</t>
+        </is>
+      </c>
+      <c r="E65" s="61" t="inlineStr">
+        <is>
+          <t>British Journal of Educational Technology</t>
+        </is>
+      </c>
+      <c r="F65" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/bjet.13613</t>
+        </is>
+      </c>
+      <c r="G65" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H65" s="59" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="59" t="n">
+        <v>7</v>
+      </c>
+      <c r="B66" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_23</t>
+        </is>
+      </c>
+      <c r="C66" s="59" t="n">
+        <v>2026</v>
+      </c>
+      <c r="D66" s="61" t="inlineStr">
+        <is>
+          <t>AI-supported higher-order thinking and EFL writing quality: A mechanism-focused study</t>
+        </is>
+      </c>
+      <c r="E66" s="61" t="inlineStr">
+        <is>
+          <t>Acta Psychologica</t>
+        </is>
+      </c>
+      <c r="F66" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.actpsy.2026.106239</t>
+        </is>
+      </c>
+      <c r="G66" s="59" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H66" s="59" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="59" t="n">
+        <v>8</v>
+      </c>
+      <c r="B67" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_231</t>
+        </is>
+      </c>
+      <c r="C67" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D67" s="61" t="inlineStr">
+        <is>
+          <t>Breaking human dominance: Investigating learners' preferences for learning feedback from generative AI and human tutors</t>
+        </is>
+      </c>
+      <c r="E67" s="61" t="inlineStr">
+        <is>
+          <t>British Journal of Educational Technology</t>
+        </is>
+      </c>
+      <c r="F67" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/bjet.13614</t>
+        </is>
+      </c>
+      <c r="G67" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H67" s="59" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="59" t="n">
+        <v>9</v>
+      </c>
+      <c r="B68" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_257</t>
+        </is>
+      </c>
+      <c r="C68" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D68" s="61" t="inlineStr">
+        <is>
+          <t>Stench of Errors or the Shine of Potential: The Challenge of (Ir)Responsible Use of ChatGPT in Speech-Language Pathology</t>
+        </is>
+      </c>
+      <c r="E68" s="61" t="inlineStr">
+        <is>
+          <t>International Journal of Language and Communication Disorders</t>
+        </is>
+      </c>
+      <c r="F68" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/1460-6984.70088</t>
+        </is>
+      </c>
+      <c r="G68" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H68" s="59" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="B69" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_277</t>
+        </is>
+      </c>
+      <c r="C69" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D69" s="61" t="inlineStr">
+        <is>
+          <t>The critical role of trust in adopting AI-powered educational technology for learning: An instrument for measuring student perceptions</t>
+        </is>
+      </c>
+      <c r="E69" s="61" t="inlineStr">
+        <is>
+          <t>Computers and Education: Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F69" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.caeai.2025.100368</t>
+        </is>
+      </c>
+      <c r="G69" s="59" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H69" s="59" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="59" t="n">
+        <v>11</v>
+      </c>
+      <c r="B70" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_296</t>
+        </is>
+      </c>
+      <c r="C70" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D70" s="61" t="inlineStr">
+        <is>
+          <t>A cross-country analysis of self-determination and continuance use intention of AI tools in business education: Does instructor support matter?</t>
+        </is>
+      </c>
+      <c r="E70" s="61" t="inlineStr">
+        <is>
+          <t>Computers and Education: Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F70" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.caeai.2025.100402</t>
+        </is>
+      </c>
+      <c r="G70" s="59" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H70" s="59" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="59" t="n">
+        <v>12</v>
+      </c>
+      <c r="B71" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_297</t>
+        </is>
+      </c>
+      <c r="C71" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D71" s="61" t="inlineStr">
+        <is>
+          <t>A comparative analysis of pre-service teachers’ readiness for AI integration</t>
+        </is>
+      </c>
+      <c r="E71" s="61" t="inlineStr">
+        <is>
+          <t>Computers and Education: Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F71" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.caeai.2025.100396</t>
+        </is>
+      </c>
+      <c r="G71" s="59" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H71" s="59" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="59" t="n">
+        <v>13</v>
+      </c>
+      <c r="B72" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_329</t>
+        </is>
+      </c>
+      <c r="C72" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D72" s="61" t="inlineStr">
+        <is>
+          <t>Shifting Dynamics: Who Holds the Reins in Decision-Making With Artificial Intelligence Tools? Perspectives of Gen Z Pre-Service Teachers</t>
+        </is>
+      </c>
+      <c r="E72" s="61" t="inlineStr">
+        <is>
+          <t>European Journal of Education</t>
+        </is>
+      </c>
+      <c r="F72" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/ejed.70053</t>
+        </is>
+      </c>
+      <c r="G72" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H72" s="59" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="59" t="n">
+        <v>14</v>
+      </c>
+      <c r="B73" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_407</t>
+        </is>
+      </c>
+      <c r="C73" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D73" s="61" t="inlineStr">
+        <is>
+          <t>Would You Trust Your GenAI Chatbot as Your School Therapist? Perspectives and Implications From Teachers and Students</t>
+        </is>
+      </c>
+      <c r="E73" s="61" t="inlineStr">
+        <is>
+          <t>Human Behavior and Emerging Technologies</t>
+        </is>
+      </c>
+      <c r="F73" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1155/hbe2/8841208</t>
+        </is>
+      </c>
+      <c r="G73" s="59" t="inlineStr">
+        <is>
+          <t>Hindawi/Wiley</t>
+        </is>
+      </c>
+      <c r="H73" s="59" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="B74" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_425</t>
+        </is>
+      </c>
+      <c r="C74" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D74" s="61" t="inlineStr">
+        <is>
+          <t>The role of over-reliance on AI in the negative consequences of student learning: The moderating effects of ethical concerns and institutional policies</t>
+        </is>
+      </c>
+      <c r="E74" s="61" t="inlineStr">
+        <is>
+          <t>Cogent Education</t>
+        </is>
+      </c>
+      <c r="F74" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/2331186x.2025.2591503</t>
+        </is>
+      </c>
+      <c r="G74" s="59" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H74" s="59" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="59" t="n">
+        <v>16</v>
+      </c>
+      <c r="B75" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_447</t>
+        </is>
+      </c>
+      <c r="C75" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D75" s="61" t="inlineStr">
+        <is>
+          <t>Beyond Teacher-Led Approaches: Student-Initiated Translanguaging With Artificial Intelligence Tools in Foreign Language Acquisition</t>
+        </is>
+      </c>
+      <c r="E75" s="61" t="inlineStr">
+        <is>
+          <t>SAGE Open</t>
+        </is>
+      </c>
+      <c r="F75" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/21582440251362998</t>
+        </is>
+      </c>
+      <c r="G75" s="59" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H75" s="59" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="59" t="n">
+        <v>17</v>
+      </c>
+      <c r="B76" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_491</t>
+        </is>
+      </c>
+      <c r="C76" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D76" s="61" t="inlineStr">
+        <is>
+          <t>Supporting learner agency in collaborative writing with generative AI</t>
+        </is>
+      </c>
+      <c r="E76" s="61" t="inlineStr">
+        <is>
+          <t>British Journal of Educational Technology</t>
+        </is>
+      </c>
+      <c r="F76" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/bjet.70015</t>
+        </is>
+      </c>
+      <c r="G76" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H76" s="59" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="59" t="n">
+        <v>18</v>
+      </c>
+      <c r="B77" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_588</t>
+        </is>
+      </c>
+      <c r="C77" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D77" s="61" t="inlineStr">
+        <is>
+          <t>Leveraging AI for Writing Instruction in EFL Classrooms: Opportunities and Challenges</t>
+        </is>
+      </c>
+      <c r="E77" s="61" t="inlineStr">
+        <is>
+          <t>Educational Process: International Journal</t>
+        </is>
+      </c>
+      <c r="F77" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.22521/edupij.2025.15.158</t>
+        </is>
+      </c>
+      <c r="G77" s="59" t="inlineStr">
+        <is>
+          <t>EDUPIJ</t>
+        </is>
+      </c>
+      <c r="H77" s="59" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="59" t="n">
+        <v>19</v>
+      </c>
+      <c r="B78" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_591</t>
+        </is>
+      </c>
+      <c r="C78" s="59" t="n">
+        <v>2025</v>
+      </c>
+      <c r="D78" s="61" t="inlineStr">
+        <is>
+          <t>Ethical considerations of AI through a socio-technical lens: insights from ELT context as a higher education system</t>
+        </is>
+      </c>
+      <c r="E78" s="61" t="inlineStr">
+        <is>
+          <t>Cogent Education</t>
+        </is>
+      </c>
+      <c r="F78" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1080/2331186x.2025.2488546</t>
+        </is>
+      </c>
+      <c r="G78" s="59" t="inlineStr">
+        <is>
+          <t>Taylor &amp; Francis</t>
+        </is>
+      </c>
+      <c r="H78" s="59" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="59" t="n">
+        <v>20</v>
+      </c>
+      <c r="B79" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_626</t>
+        </is>
+      </c>
+      <c r="C79" s="59" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D79" s="61" t="inlineStr">
+        <is>
+          <t>Self-directed use of machine translation among language learners: Does it lead to disruptive L2 avoidance?</t>
+        </is>
+      </c>
+      <c r="E79" s="61" t="inlineStr">
+        <is>
+          <t>Foreign Language Annals</t>
+        </is>
+      </c>
+      <c r="F79" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/flan.12768</t>
+        </is>
+      </c>
+      <c r="G79" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H79" s="59" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="59" t="n">
+        <v>21</v>
+      </c>
+      <c r="B80" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_631</t>
+        </is>
+      </c>
+      <c r="C80" s="59" t="n">
+        <v>2024</v>
+      </c>
+      <c r="D80" s="61" t="inlineStr">
+        <is>
+          <t>Meaningful Communication but not Superficial Anthropomorphism Facilitates Human-Automation Trust Calibration: The Human-Automation Trust Expectation Model (HATEM)</t>
+        </is>
+      </c>
+      <c r="E80" s="61" t="inlineStr">
+        <is>
+          <t>Human Factors</t>
+        </is>
+      </c>
+      <c r="F80" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1177/00187208231218156</t>
+        </is>
+      </c>
+      <c r="G80" s="59" t="inlineStr">
+        <is>
+          <t>SAGE</t>
+        </is>
+      </c>
+      <c r="H80" s="59" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="59" t="n">
+        <v>22</v>
+      </c>
+      <c r="B81" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_822</t>
+        </is>
+      </c>
+      <c r="C81" s="59" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D81" s="61" t="inlineStr">
+        <is>
+          <t>Teachers' trust in AI-powered educational technology and a professional development program to improve it</t>
+        </is>
+      </c>
+      <c r="E81" s="61" t="inlineStr">
+        <is>
+          <t>British Journal of Educational Technology</t>
+        </is>
+      </c>
+      <c r="F81" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1111/bjet.13232</t>
+        </is>
+      </c>
+      <c r="G81" s="59" t="inlineStr">
+        <is>
+          <t>Wiley</t>
+        </is>
+      </c>
+      <c r="H81" s="59" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="59" t="n">
+        <v>23</v>
+      </c>
+      <c r="B82" s="60" t="inlineStr">
+        <is>
+          <t>SCOPUS_834</t>
+        </is>
+      </c>
+      <c r="C82" s="59" t="n">
+        <v>2022</v>
+      </c>
+      <c r="D82" s="61" t="inlineStr">
+        <is>
+          <t>Explainable Artificial Intelligence in education</t>
+        </is>
+      </c>
+      <c r="E82" s="61" t="inlineStr">
+        <is>
+          <t>Computers and Education: Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="F82" s="62" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1016/j.caeai.2022.100074</t>
+        </is>
+      </c>
+      <c r="G82" s="59" t="inlineStr">
+        <is>
+          <t>Elsevier</t>
+        </is>
+      </c>
+      <c r="H82" s="59" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A2:H56"/>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A58:H58"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
   <dataValidations count="1">
@@ -51696,6 +52583,29 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F54" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F55" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F56" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F60" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F61" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F62" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F63" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F64" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F65" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F66" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F67" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F68" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F69" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F70" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F71" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F72" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F73" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F74" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F75" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F76" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F77" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F78" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F79" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F80" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F81" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F82" r:id="rId75"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add Abdalla (2024) paper and complete full-text coding
- Add Paper #129 (CT_1): "Higher education students' trust and use
  of ChatGPT: empirical evidence" (Abdalla, 2024, IJTEL)
- Source: citation-tracked from Zotero AI trust3 library
- Updated sheets: ⓪ 논문 번호표, ① 스크리닝, ② 포함 논문, ③ Full-text 코딩
- Complete 32-column coding: empirical/quantitative, UTAUT+EVT
  framework, trust as mediator (3-item scale), n=127 PTUK students
- Relevance score: 2 (trust studied but no calibration angle)
- Included via BR2 (UTAUT + β reported) and BR5 (3-item trust scale)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resource/TCS_screening_coding_v1.xlsx
+++ b/resource/TCS_screening_coding_v1.xlsx
@@ -350,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -564,6 +564,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -931,7 +951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H129"/>
+  <dimension ref="A1:H130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5839,6 +5859,44 @@
       <c r="H129" s="70" t="inlineStr">
         <is>
           <t>✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="86" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="87" t="inlineStr">
+        <is>
+          <t>CT_1</t>
+        </is>
+      </c>
+      <c r="C130" s="88" t="inlineStr">
+        <is>
+          <t>Abdalla</t>
+        </is>
+      </c>
+      <c r="D130" s="89" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E130" s="90" t="inlineStr">
+        <is>
+          <t>Higher education students' trust and use of ChatGPT: empirical evidence</t>
+        </is>
+      </c>
+      <c r="F130" s="90" t="inlineStr">
+        <is>
+          <t>International Journal of Technology Enhanced Learning</t>
+        </is>
+      </c>
+      <c r="G130" s="91" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/IJTEL.2024.10061581</t>
+        </is>
+      </c>
+      <c r="H130" s="70" t="inlineStr">
+        <is>
+          <t>📄</t>
         </is>
       </c>
     </row>
@@ -5982,7 +6040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K801"/>
+  <dimension ref="A1:K802"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -47833,6 +47891,55 @@
       <c r="K801" s="33" t="inlineStr">
         <is>
           <t>Investigates L2 learners' perceptions of ChatGPT interference with voice in academic writing; trust not a dedicated measured construct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="5" t="n">
+        <v>800</v>
+      </c>
+      <c r="B802" s="5" t="inlineStr">
+        <is>
+          <t>CT_1</t>
+        </is>
+      </c>
+      <c r="C802" s="5" t="inlineStr">
+        <is>
+          <t>Higher education students' trust and use of ChatGPT: empirical evidence</t>
+        </is>
+      </c>
+      <c r="D802" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="E802" s="5" t="inlineStr">
+        <is>
+          <t>International Journal of Technology Enhanced Learning</t>
+        </is>
+      </c>
+      <c r="F802" s="6" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/IJTEL.2024.10061581</t>
+        </is>
+      </c>
+      <c r="G802" s="5" t="inlineStr">
+        <is>
+          <t>citation_tracked</t>
+        </is>
+      </c>
+      <c r="H802" s="7" t="inlineStr">
+        <is>
+          <t>This paper combines a modified version of the unified theory of acceptance and use of technology (UATAU) with the expectancy value theory (EVT) to examine the variables that influence higher education students' trust and use of ChatGPT. The quantitative method was used, with a structured questionnaire developed to collect data from respondents, which was then analysed using Smart PLS 4. According to the findings, perceived mobility influenced performance and effort expectancy, while social influence and performance expectancy determined students' trust. The three predicted elements that influenced ChatGPT adoption were perceived learning gains, perceived risks, and trust in ChatGPT.</t>
+        </is>
+      </c>
+      <c r="I802" s="92" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="J802" s="53" t="n"/>
+      <c r="K802" s="7" t="inlineStr">
+        <is>
+          <t>Include via BR2 (UTAUT with trust as mediator, β reported) and BR5 (3-item trust subscale). Citation-tracked from AI trust3 Zotero library.</t>
         </is>
       </c>
     </row>
@@ -48644,7 +48751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M130"/>
+  <dimension ref="A1:M131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -53956,6 +54063,47 @@
       <c r="K130" s="46" t="n"/>
       <c r="L130" s="46" t="n"/>
       <c r="M130" s="46" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="85" t="n">
+        <v>129</v>
+      </c>
+      <c r="B131" s="46" t="n">
+        <v>129</v>
+      </c>
+      <c r="C131" s="46" t="inlineStr">
+        <is>
+          <t>CT_1</t>
+        </is>
+      </c>
+      <c r="D131" s="5" t="inlineStr">
+        <is>
+          <t>Higher education students' trust and use of ChatGPT: empirical evidence</t>
+        </is>
+      </c>
+      <c r="E131" s="46" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F131" s="46" t="inlineStr">
+        <is>
+          <t>International Journal of Technology Enhanced Learning</t>
+        </is>
+      </c>
+      <c r="G131" s="47" t="inlineStr">
+        <is>
+          <t>📄</t>
+        </is>
+      </c>
+      <c r="H131" s="46" t="inlineStr">
+        <is>
+          <t>Abdalla, R.A.M.</t>
+        </is>
+      </c>
+      <c r="I131" s="46" t="n"/>
+      <c r="J131" s="46" t="n"/>
+      <c r="K131" s="46" t="n"/>
+      <c r="L131" s="46" t="n"/>
+      <c r="M131" s="46" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -54329,7 +54477,158 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
+    <row r="3">
+      <c r="A3" s="93" t="n">
+        <v>129</v>
+      </c>
+      <c r="B3" s="93" t="n">
+        <v>129</v>
+      </c>
+      <c r="C3" s="93" t="inlineStr">
+        <is>
+          <t>CT_1</t>
+        </is>
+      </c>
+      <c r="D3" s="93" t="inlineStr">
+        <is>
+          <t>Abdalla, R.A.M.</t>
+        </is>
+      </c>
+      <c r="E3" s="93" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F3" s="93" t="inlineStr">
+        <is>
+          <t>Higher education students' trust and use of ChatGPT: empirical evidence</t>
+        </is>
+      </c>
+      <c r="G3" s="93" t="inlineStr">
+        <is>
+          <t>International Journal of Technology Enhanced Learning</t>
+        </is>
+      </c>
+      <c r="H3" s="93" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1504/IJTEL.2024.10061581</t>
+        </is>
+      </c>
+      <c r="I3" s="93" t="inlineStr">
+        <is>
+          <t>empirical</t>
+        </is>
+      </c>
+      <c r="J3" s="93" t="inlineStr">
+        <is>
+          <t>quantitative</t>
+        </is>
+      </c>
+      <c r="K3" s="93" t="inlineStr">
+        <is>
+          <t>Higher education; Palestine Technical University-Kadoorie (PTUK); undergraduate/postgraduate students</t>
+        </is>
+      </c>
+      <c r="L3" s="93" t="inlineStr">
+        <is>
+          <t>ChatGPT</t>
+        </is>
+      </c>
+      <c r="M3" s="93" t="n">
+        <v>127</v>
+      </c>
+      <c r="N3" s="93" t="inlineStr">
+        <is>
+          <t>implicit</t>
+        </is>
+      </c>
+      <c r="O3" s="93" t="inlineStr">
+        <is>
+          <t>trust_in_AI</t>
+        </is>
+      </c>
+      <c r="P3" s="93" t="inlineStr">
+        <is>
+          <t>unidimensional</t>
+        </is>
+      </c>
+      <c r="Q3" s="93" t="inlineStr">
+        <is>
+          <t>UTAUT + EVT</t>
+        </is>
+      </c>
+      <c r="R3" s="93" t="inlineStr">
+        <is>
+          <t>applied</t>
+        </is>
+      </c>
+      <c r="S3" s="93" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="T3" s="93" t="inlineStr">
+        <is>
+          <t>self-report</t>
+        </is>
+      </c>
+      <c r="U3" s="93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V3" s="93" t="inlineStr">
+        <is>
+          <t>Custom 3-item scale (Trust1-3); adapted from prior literature</t>
+        </is>
+      </c>
+      <c r="W3" s="93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="X3" s="93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Y3" s="93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="Z3" s="93" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="AA3" s="93" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AB3" s="93" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="AC3" s="93" t="inlineStr">
+        <is>
+          <t>Study focuses on trust antecedents (performance expectancy β=0.432, social influence β=0.341, effort expectancy n.s.) and trust→use path (β=0.273). Trust measured as level only via 3 Likert items (CR=0.832, AVE=0.630). No discussion of calibration, overtrust/undertrust, or oversight. R²(trust)=43.5%, R²(use)=38.5%. UTAUT+EVT model. Perceived risks negatively predict use (β=-0.225).</t>
+        </is>
+      </c>
+      <c r="AD3" s="93" t="n">
+        <v>2</v>
+      </c>
+      <c r="AE3" s="93" t="inlineStr">
+        <is>
+          <t>Performance expectancy and social influence positively predict trust in ChatGPT; effort expectancy does not. Trust, perceived benefits, and perceived risks predict ChatGPT use. Modified UTAUT+EVT model explains 43.5% of trust variance and 38.5% of use variance. Perceived mobility is key external antecedent.</t>
+        </is>
+      </c>
+      <c r="AF3" s="93" t="inlineStr">
+        <is>
+          <t>Included via BR2 (UTAUT with trust as mediator, β reported) and BR5 (3-item trust subscale). Single-institution study in Palestine. Survey-based cross-sectional design. PLS-SEM analysis via SmartPLS 4.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="AC1:AE1"/>

</xml_diff>